<commit_message>
Replace repository contents with latest local project
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/advanced_tables.xlsx
+++ b/outputs/advanced_tables.xlsx
@@ -10,8 +10,8 @@
     <sheet name="p控制图" sheetId="1" r:id="rId1"/>
     <sheet name="商家Wilson区间" sheetId="2" r:id="rId2"/>
     <sheet name="穿戴类对比" sheetId="3" r:id="rId3"/>
-    <sheet name="抽检增益曲线" sheetId="4" r:id="rId4"/>
-    <sheet name="风险模型回测" sheetId="5" r:id="rId5"/>
+    <sheet name="增益曲线" sheetId="4" r:id="rId4"/>
+    <sheet name="商家分层回测" sheetId="5" r:id="rId5"/>
     <sheet name="情景测算" sheetId="6" r:id="rId6"/>
     <sheet name="敏感性" sheetId="7" r:id="rId7"/>
   </sheets>
@@ -1096,7 +1096,7 @@
     <t>商家 × 品类风险分</t>
   </si>
   <si>
-    <t>出库复核：多件订单优先（少件问题）</t>
+    <t>出库复核：多件订单优先</t>
   </si>
   <si>
     <t>训练窗口</t>
@@ -1111,13 +1111,13 @@
     <t>商家数</t>
   </si>
   <si>
-    <t>训练期客诉率</t>
-  </si>
-  <si>
-    <t>检验期客诉率</t>
-  </si>
-  <si>
-    <t>检验期平台</t>
+    <t>训练期品质客诉率</t>
+  </si>
+  <si>
+    <t>检验期品质客诉率</t>
+  </si>
+  <si>
+    <t>检验期商家基准品质客诉率</t>
   </si>
   <si>
     <t>检验期倍数</t>
@@ -1144,7 +1144,7 @@
     <t>2018-03~2018-08</t>
   </si>
   <si>
-    <t>不平滑：原始客诉率 ≥ 2 倍</t>
+    <t>对照：未平滑的品质客诉率 ≥ 商家基准品质客诉率 × 2</t>
   </si>
   <si>
     <t>情景</t>
@@ -1195,13 +1195,13 @@
     <t>影响幅度</t>
   </si>
   <si>
-    <t>A 多件订单少件客诉降幅</t>
-  </si>
-  <si>
-    <t>B 风险商家客诉降幅</t>
-  </si>
-  <si>
-    <t>C 3C/钟表假货与货不对板降幅</t>
+    <t>举措 A 降幅</t>
+  </si>
+  <si>
+    <t>举措 B 降幅</t>
+  </si>
+  <si>
+    <t>举措 C 降幅</t>
   </si>
 </sst>
 </file>
@@ -11056,10 +11056,10 @@
         <v>0.05007824726134585</v>
       </c>
       <c r="C3">
-        <v>0.08137715179968701</v>
+        <v>0.08059467918622848</v>
       </c>
       <c r="D3">
-        <v>0.08450704225352113</v>
+        <v>0.08528951486697965</v>
       </c>
       <c r="E3">
         <v>0.386013986013986</v>
@@ -11073,10 +11073,10 @@
         <v>0.1025039123630673</v>
       </c>
       <c r="C4">
-        <v>0.1330203442879499</v>
+        <v>0.1377151799687011</v>
       </c>
       <c r="D4">
-        <v>0.1580594679186229</v>
+        <v>0.1572769953051643</v>
       </c>
       <c r="E4">
         <v>0.7538461538461538</v>
@@ -11110,7 +11110,7 @@
         <v>0.3028169014084507</v>
       </c>
       <c r="D6">
-        <v>0.3004694835680751</v>
+        <v>0.3020344287949921</v>
       </c>
       <c r="E6">
         <v>0.7902097902097902</v>
@@ -11127,7 +11127,7 @@
         <v>0.3575899843505477</v>
       </c>
       <c r="D7">
-        <v>0.3677621283255086</v>
+        <v>0.3669796557120501</v>
       </c>
       <c r="E7">
         <v>0.7986013986013986</v>
@@ -11141,7 +11141,7 @@
         <v>0.2856025039123631</v>
       </c>
       <c r="C8">
-        <v>0.405320813771518</v>
+        <v>0.4045383411580595</v>
       </c>
       <c r="D8">
         <v>0.4241001564945227</v>
@@ -11158,7 +11158,7 @@
         <v>0.3325508607198748</v>
       </c>
       <c r="C9">
-        <v>0.4514866979655712</v>
+        <v>0.4538341158059468</v>
       </c>
       <c r="D9">
         <v>0.4687010954616588</v>
@@ -11175,10 +11175,10 @@
         <v>0.3857589984350548</v>
       </c>
       <c r="C10">
-        <v>0.5039123630672926</v>
+        <v>0.4906103286384976</v>
       </c>
       <c r="D10">
-        <v>0.5172143974960877</v>
+        <v>0.5164319248826291</v>
       </c>
       <c r="E10">
         <v>0.8363636363636363</v>
@@ -11192,10 +11192,10 @@
         <v>0.431924882629108</v>
       </c>
       <c r="C11">
-        <v>0.5438184663536776</v>
+        <v>0.5391236306729265</v>
       </c>
       <c r="D11">
-        <v>0.5586854460093896</v>
+        <v>0.5610328638497653</v>
       </c>
       <c r="E11">
         <v>0.8475524475524475</v>
@@ -11226,7 +11226,7 @@
         <v>0.5328638497652582</v>
       </c>
       <c r="C13">
-        <v>0.6353677621283255</v>
+        <v>0.6314553990610329</v>
       </c>
       <c r="D13">
         <v>0.6799687010954617</v>
@@ -11243,10 +11243,10 @@
         <v>0.582942097026604</v>
       </c>
       <c r="C14">
-        <v>0.7136150234741784</v>
+        <v>0.7128325508607198</v>
       </c>
       <c r="D14">
-        <v>0.7222222222222222</v>
+        <v>0.7253521126760564</v>
       </c>
       <c r="E14">
         <v>0.8839160839160839</v>
@@ -11260,7 +11260,7 @@
         <v>0.6298904538341158</v>
       </c>
       <c r="C15">
-        <v>0.7644757433489828</v>
+        <v>0.7629107981220657</v>
       </c>
       <c r="D15">
         <v>0.7621283255086072</v>
@@ -11277,7 +11277,7 @@
         <v>0.6823161189358372</v>
       </c>
       <c r="C16">
-        <v>0.798904538341158</v>
+        <v>0.797339593114241</v>
       </c>
       <c r="D16">
         <v>0.8161189358372457</v>
@@ -11311,7 +11311,7 @@
         <v>0.7848200312989045</v>
       </c>
       <c r="C18">
-        <v>0.863849765258216</v>
+        <v>0.86697965571205</v>
       </c>
       <c r="D18">
         <v>0.8802816901408451</v>
@@ -11345,10 +11345,10 @@
         <v>0.8826291079812206</v>
       </c>
       <c r="C20">
-        <v>0.9491392801251957</v>
+        <v>0.9522691705790297</v>
       </c>
       <c r="D20">
-        <v>0.9522691705790297</v>
+        <v>0.9507042253521126</v>
       </c>
       <c r="E20">
         <v>0.9734265734265735</v>
@@ -11362,7 +11362,7 @@
         <v>0.9420970266040689</v>
       </c>
       <c r="C21">
-        <v>0.9773082942097027</v>
+        <v>0.9780907668231612</v>
       </c>
       <c r="D21">
         <v>0.9804381846635368</v>

</xml_diff>